<commit_message>
commit week 4 material
</commit_message>
<xml_diff>
--- a/Week 3/python_Excel.xlsx
+++ b/Week 3/python_Excel.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop W11\working_folder\Personales\Upright\Data_Science\Instructor_material\wk3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ab76ec252c957cd7/Desktop/data_bootcamp_folder/instructor_ref/instructor_ref/Week 3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BED6573B-4012-47AB-BB4C-58CBA0164927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{BED6573B-4012-47AB-BB4C-58CBA0164927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7387BBE8-5149-4595-AC77-160A04A6338E}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{8516C1E8-9EA0-482A-91C9-2CE1A2DB7C28}"/>
+    <workbookView xWindow="3790" yWindow="1470" windowWidth="19570" windowHeight="12620" xr2:uid="{8516C1E8-9EA0-482A-91C9-2CE1A2DB7C28}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -184,7 +184,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -872,15 +872,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>173991</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>135891</xdr:rowOff>
+      <xdr:colOff>93300</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>118350</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>576581</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>180909</xdr:rowOff>
+      <xdr:colOff>495890</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>163368</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -903,8 +903,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7603491" y="5139691"/>
-          <a:ext cx="3450590" cy="1886518"/>
+          <a:off x="7632609" y="5159759"/>
+          <a:ext cx="3454800" cy="1869327"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -916,15 +916,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>3810</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:colOff>73976</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>151382</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>340063</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>99060</xdr:rowOff>
+      <xdr:colOff>410229</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>155193</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -947,8 +947,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7433310" y="8045450"/>
-          <a:ext cx="3993853" cy="1477010"/>
+          <a:off x="7613285" y="8111686"/>
+          <a:ext cx="3998905" cy="1463258"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1278,16 +1278,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F42948C-A579-4CF2-B45D-6BC7113BD4CF}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="30.109375" customWidth="1"/>
-    <col min="2" max="2" width="17.21875" customWidth="1"/>
-    <col min="3" max="3" width="16.88671875" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" customWidth="1"/>
-    <col min="6" max="6" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.08984375" customWidth="1"/>
+    <col min="2" max="2" width="17.1796875" customWidth="1"/>
+    <col min="3" max="3" width="16.90625" customWidth="1"/>
+    <col min="4" max="4" width="13.08984375" customWidth="1"/>
+    <col min="6" max="6" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="41.4">
+    <row r="1" spans="1:3" ht="28">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1298,7 +1298,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="26.4">
+    <row r="2" spans="1:3" ht="25">
       <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:3" ht="26.4">
+    <row r="3" spans="1:3" ht="25">
       <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:3" ht="26.4">
+    <row r="4" spans="1:3" ht="25">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C4" s="1"/>
     </row>
-    <row r="7" spans="1:3" ht="171.6">
+    <row r="7" spans="1:3" ht="150">
       <c r="A7" s="7" t="s">
         <v>9</v>
       </c>

</xml_diff>